<commit_message>
v1.4: Bitacora de control de versiones finalizada por Gabriela Torres
</commit_message>
<xml_diff>
--- a/plantillas control de versiones.xlsx
+++ b/plantillas control de versiones.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11700"/>
+    <workbookView windowWidth="27945" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="89">
   <si>
     <t>Proyecto</t>
   </si>
@@ -82,24 +82,24 @@
     <t>v1.0</t>
   </si>
   <si>
-    <t>Juan Pérez</t>
-  </si>
-  <si>
-    <t>Creación inicial del archivo</t>
+    <t>17/07/2026</t>
+  </si>
+  <si>
+    <t>Gabriela Torres</t>
+  </si>
+  <si>
+    <t>Creación inicial del archivo Login.java</t>
   </si>
   <si>
     <t>Creación</t>
   </si>
   <si>
-    <t>Docente</t>
+    <t>profesor</t>
   </si>
   <si>
     <t>v1.1</t>
   </si>
   <si>
-    <t>María López</t>
-  </si>
-  <si>
     <t>Se agregó validación del usuario</t>
   </si>
   <si>
@@ -109,9 +109,6 @@
     <t>v1.2</t>
   </si>
   <si>
-    <t>Carlos Díaz</t>
-  </si>
-  <si>
     <t>Corrección de errores en el login</t>
   </si>
   <si>
@@ -121,16 +118,10 @@
     <t>v1.3</t>
   </si>
   <si>
-    <t>Ana Ruiz</t>
-  </si>
-  <si>
     <t>Se agregó recuperación de contraseña</t>
   </si>
   <si>
     <t>Nueva funcionalidad</t>
-  </si>
-  <si>
-    <t>Pedro Silva</t>
   </si>
   <si>
     <t>Optimización del proceso de autenticación</t>
@@ -317,7 +308,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -348,13 +339,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -499,7 +483,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -575,12 +559,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -814,152 +792,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -982,6 +960,9 @@
     </xf>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1520,31 +1501,31 @@
       <c r="B12" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="14">
-        <v>46213</v>
+      <c r="C12" s="15" t="s">
+        <v>17</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="13" t="s">
         <v>18</v>
       </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
       <c r="F12" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" ht="30" spans="2:7">
       <c r="B13" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C13" s="14">
-        <v>46213</v>
+        <v>22</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>17</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>23</v>
@@ -1553,72 +1534,72 @@
         <v>24</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" ht="30" spans="2:7">
       <c r="B14" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="14">
-        <v>46214</v>
+      <c r="C14" s="15" t="s">
+        <v>17</v>
       </c>
       <c r="D14" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="F14" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="13" t="s">
-        <v>28</v>
-      </c>
       <c r="G14" s="13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" ht="30" spans="2:7">
       <c r="B15" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="14">
-        <v>46214</v>
-      </c>
-      <c r="D15" s="13" t="s">
+      <c r="F15" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>32</v>
-      </c>
       <c r="G15" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" ht="30" spans="2:7">
       <c r="B16" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="14">
-        <v>46215</v>
+      <c r="C16" s="15" t="s">
+        <v>17</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="2:7">
       <c r="B19" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="2:7">
@@ -1632,13 +1613,13 @@
         <v>12</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="2:7">
@@ -1649,16 +1630,16 @@
         <v>46213</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>3</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" ht="30" spans="2:7">
@@ -1669,7 +1650,7 @@
         <v>46213</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>3</v>
@@ -1678,27 +1659,27 @@
         <v>23</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" ht="30" spans="2:7">
       <c r="B23" s="13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C23" s="14">
         <v>46214</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>3</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="2:7">
@@ -1706,7 +1687,7 @@
     </row>
     <row r="27" spans="2:7">
       <c r="B27" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="2:7">
@@ -1714,16 +1695,16 @@
         <v>11</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" ht="30" spans="2:7">
@@ -1734,29 +1715,29 @@
         <v>3</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" spans="2:4">
       <c r="B33" s="6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="2:4">
       <c r="B34" s="11" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>11</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="35" ht="30" spans="2:4">
@@ -1767,7 +1748,7 @@
         <v>46215</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1808,37 +1789,37 @@
   <sheetData>
     <row r="3" spans="2:13">
       <c r="E3" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="2:13">
       <c r="B4" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="2:13">
       <c r="E5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="2:13">
       <c r="E6" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J6" s="4">
         <v>46023</v>
@@ -1855,173 +1836,173 @@
     </row>
     <row r="7" spans="2:13">
       <c r="E7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H7" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>71</v>
-      </c>
       <c r="K7" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="2:13">
       <c r="H8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="L8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="M8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="2:13">
       <c r="H9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="L9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="M9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="2:13">
       <c r="B10" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="J10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="M10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="2:13">
       <c r="B11" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="J11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="L11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="2:13">
       <c r="B12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="J12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="L12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="M12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="2:13">
       <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" t="s">
         <v>75</v>
-      </c>
-      <c r="C13" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="14" spans="2:13">
       <c r="B14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="2:13">
       <c r="B15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="J15" s="4">
         <v>46357</v>
@@ -2029,71 +2010,71 @@
     </row>
     <row r="16" spans="2:13">
       <c r="G16" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="J16" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="17" spans="7:12">
       <c r="H17" s="9" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I17" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="J17" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="7:12">
       <c r="H18" s="9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="J18" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="7:12">
       <c r="G19" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I19" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J19" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="7:12">
       <c r="H20" s="9" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="J20" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="7:12">
       <c r="H21" s="9" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I21" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J21" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="7:12">
@@ -2112,66 +2093,66 @@
     </row>
     <row r="25" ht="26.25" spans="7:12">
       <c r="G25" s="10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="7:12">
       <c r="G26" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H26" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I26" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="7:12">
       <c r="G27" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="H27" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="J27" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="K27" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="7:12">
       <c r="G28" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="H28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I28" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="7:12">
       <c r="G29" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H29" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I29" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>